<commit_message>
committees.html: display Country alongside University in all sections
</commit_message>
<xml_diff>
--- a/ainetec2027.xlsx
+++ b/ainetec2027.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anas\Documents\GitHub\AINTEC-website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDFAFB5F-48D4-4BD6-992D-79E538A34D7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{126F5FB0-5EBE-43C7-9212-4B71CCDFCF79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{EF8DF1C2-0E33-41ED-BB28-B7B3BA38219D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{EF8DF1C2-0E33-41ED-BB28-B7B3BA38219D}"/>
   </bookViews>
   <sheets>
     <sheet name="Honorary Committee" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="16">
   <si>
     <t>Nom</t>
   </si>
@@ -70,6 +70,12 @@
   </si>
   <si>
     <t>Co-Chairs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Morocco </t>
+  </si>
+  <si>
+    <t>Country</t>
   </si>
 </sst>
 </file>
@@ -958,6 +964,9 @@
       <c r="C1" t="s">
         <v>9</v>
       </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -969,7 +978,9 @@
       <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="1"/>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -978,7 +989,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52BED034-24DB-4F53-80DA-5A9D61FF4369}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -987,7 +998,7 @@
     <col min="4" max="4" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1001,10 +1012,13 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1018,10 +1032,13 @@
         <v>8</v>
       </c>
       <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1035,6 +1052,9 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1048,14 +1068,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85AF5B3B-0FE8-4F76-8139-65C6018633CF}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="27.33203125" customWidth="1"/>
     <col min="4" max="4" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1068,8 +1088,11 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1081,6 +1104,9 @@
       </c>
       <c r="D2" s="1" t="s">
         <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1093,7 +1119,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27BDA498-39C4-4CD1-8FD2-A7BB7C7DEB39}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.5546875" customWidth="1"/>
@@ -1102,7 +1128,7 @@
     <col min="5" max="5" width="17.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1115,8 +1141,11 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1128,6 +1157,9 @@
       </c>
       <c r="D2" s="1" t="s">
         <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>